<commit_message>
added readme files for information on OSF and corrected a typo in the codebook
</commit_message>
<xml_diff>
--- a/results/02_revision_1/codebooks/codebook_aggregated_results.xlsx
+++ b/results/02_revision_1/codebooks/codebook_aggregated_results.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CBE2088-994F-49CC-9184-5DABCF9CD5D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BA76C69-AA70-4C71-A489-C9DE55BE5FFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="205">
   <si>
     <t>Variable Name</t>
   </si>
@@ -274,15 +274,9 @@
     <t>most negative person-level difference (minimum person-level difference) (person-level difference was calculated per participant across replications)</t>
   </si>
   <si>
-    <t>ID of participant with the most positive person-level difference (maximum person-level difference) (person-level difference was calculated per participant across replications)</t>
-  </si>
-  <si>
     <t>most positive person-level difference (maximum person-level difference) (person-level difference was calculated per participant across replications)</t>
   </si>
   <si>
-    <t>ID of participant with the most negative person-level difference (minimum person-level difference) (person-level difference was calculated per participant across replications)</t>
-  </si>
-  <si>
     <t>person_diff.z</t>
   </si>
   <si>
@@ -308,12 +302,6 @@
   </si>
   <si>
     <t>median person-level difference ("bias") (for Fisher's Z-transformed ICCs) across participants (person-level difference was calculated per participant across replications)</t>
-  </si>
-  <si>
-    <t>ID of participant with the most negative person-level difference (for Fisher's Z-transformed ICCs) (minimum person-level difference) (person-level difference was calculated per participant across replications)</t>
-  </si>
-  <si>
-    <t>ID of participant with the most positive person-level difference (for Fisher's Z-transformed ICCs) (maximum person-level difference) (person-level difference was calculated per participant across replications)</t>
   </si>
   <si>
     <t>most negative person-level difference (minimum person-level difference) (for Fisher's Z-transformed ICCs) (person-level difference was calculated per participant across replications)</t>
@@ -647,6 +635,21 @@
   </si>
   <si>
     <t>maximum number of upper bound estimation problems (ICCs &gt;= +1 that cannot be Fisher's Z-transformed) across replications for a given condition</t>
+  </si>
+  <si>
+    <t>index of participant with the most negative person-level difference (minimum person-level difference) (person-level difference was calculated per participant across replications)</t>
+  </si>
+  <si>
+    <t>index of participant with the most positive person-level difference (maximum person-level difference) (person-level difference was calculated per participant across replications)</t>
+  </si>
+  <si>
+    <t>index of participant with the most negative person-level difference (for Fisher's Z-transformed ICCs) (minimum person-level difference) (person-level difference was calculated per participant across replications)</t>
+  </si>
+  <si>
+    <t>index of participant with the most positive person-level difference (for Fisher's Z-transformed ICCs) (maximum person-level difference) (person-level difference was calculated per participant across replications)</t>
+  </si>
+  <si>
+    <t>index = position in the vector with person-level differences (all vectors are in the same order)</t>
   </si>
 </sst>
 </file>
@@ -1021,30 +1024,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D186"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="57.109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="45.88671875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="65.33203125" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="11.44140625" style="1"/>
+    <col min="1" max="1" width="22.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="57.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="45.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="65.28515625" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
     </row>
-    <row r="2" spans="1:4" s="5" customFormat="1" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" s="5" customFormat="1" ht="58.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
     </row>
-    <row r="4" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
@@ -1055,21 +1058,21 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" s="6" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" s="6" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
     </row>
-    <row r="6" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
     </row>
-    <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
@@ -1078,7 +1081,7 @@
       </c>
       <c r="C7" s="2"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -1087,7 +1090,7 @@
       </c>
       <c r="C8" s="2"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
@@ -1096,42 +1099,42 @@
       </c>
       <c r="C9" s="2"/>
     </row>
-    <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="C10" s="2"/>
-    </row>
-    <row r="11" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="C11" s="2"/>
-    </row>
-    <row r="12" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+      <c r="C12" s="2"/>
+    </row>
+    <row r="13" spans="1:4" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
         <v>103</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C12" s="2"/>
-    </row>
-    <row r="13" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="8" t="s">
-        <v>107</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
       <c r="D13" s="8"/>
     </row>
-    <row r="14" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>4</v>
       </c>
@@ -1140,7 +1143,7 @@
       </c>
       <c r="C14" s="2"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>3</v>
       </c>
@@ -1149,7 +1152,7 @@
       </c>
       <c r="C15" s="2"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>5</v>
       </c>
@@ -1158,42 +1161,42 @@
       </c>
       <c r="C16" s="2"/>
     </row>
-    <row r="17" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="C17" s="2"/>
-    </row>
-    <row r="18" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
+      <c r="C18" s="2"/>
+    </row>
+    <row r="19" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="C18" s="2"/>
-    </row>
-    <row r="19" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="8" t="s">
         <v>110</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="C19" s="2"/>
-    </row>
-    <row r="20" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="8" t="s">
-        <v>114</v>
       </c>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
       <c r="D20" s="8"/>
     </row>
-    <row r="21" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
@@ -1202,7 +1205,7 @@
       </c>
       <c r="C21" s="2"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>3</v>
       </c>
@@ -1211,7 +1214,7 @@
       </c>
       <c r="C22" s="2"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>5</v>
       </c>
@@ -1220,42 +1223,42 @@
       </c>
       <c r="C23" s="2"/>
     </row>
-    <row r="24" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C24" s="2"/>
     </row>
-    <row r="25" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C25" s="2"/>
     </row>
-    <row r="26" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C26" s="2"/>
     </row>
-    <row r="27" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
       <c r="D27" s="8"/>
     </row>
-    <row r="28" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>4</v>
       </c>
@@ -1264,7 +1267,7 @@
       </c>
       <c r="C28" s="2"/>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>3</v>
       </c>
@@ -1273,7 +1276,7 @@
       </c>
       <c r="C29" s="2"/>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>5</v>
       </c>
@@ -1282,42 +1285,42 @@
       </c>
       <c r="C30" s="2"/>
     </row>
-    <row r="31" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C31" s="2"/>
+    </row>
+    <row r="32" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="C32" s="2"/>
+    </row>
+    <row r="33" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C33" s="2"/>
+    </row>
+    <row r="34" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="8" t="s">
         <v>122</v>
-      </c>
-      <c r="C31" s="2"/>
-    </row>
-    <row r="32" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="C32" s="2"/>
-    </row>
-    <row r="33" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="C33" s="2"/>
-    </row>
-    <row r="34" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="8" t="s">
-        <v>126</v>
       </c>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
       <c r="D34" s="8"/>
     </row>
-    <row r="35" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>4</v>
       </c>
@@ -1326,7 +1329,7 @@
       </c>
       <c r="C35" s="2"/>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>3</v>
       </c>
@@ -1335,7 +1338,7 @@
       </c>
       <c r="C36" s="2"/>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>5</v>
       </c>
@@ -1344,34 +1347,34 @@
       </c>
       <c r="C37" s="2"/>
     </row>
-    <row r="38" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C38" s="2"/>
+    </row>
+    <row r="39" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B38" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="C38" s="2"/>
-    </row>
-    <row r="39" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A39" s="1" t="s">
+      <c r="C39" s="2"/>
+    </row>
+    <row r="40" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B40" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B39" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="C39" s="2"/>
-    </row>
-    <row r="40" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A40" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>132</v>
-      </c>
       <c r="C40" s="2"/>
     </row>
-    <row r="41" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
         <v>9</v>
       </c>
@@ -1379,7 +1382,7 @@
       <c r="C41" s="8"/>
       <c r="D41" s="8"/>
     </row>
-    <row r="42" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>4</v>
       </c>
@@ -1388,7 +1391,7 @@
       </c>
       <c r="C42" s="2"/>
     </row>
-    <row r="43" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>3</v>
       </c>
@@ -1397,7 +1400,7 @@
       </c>
       <c r="C43" s="2"/>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>5</v>
       </c>
@@ -1406,7 +1409,7 @@
       </c>
       <c r="C44" s="2"/>
     </row>
-    <row r="45" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>39</v>
       </c>
@@ -1415,7 +1418,7 @@
       </c>
       <c r="C45" s="2"/>
     </row>
-    <row r="46" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>40</v>
       </c>
@@ -1424,7 +1427,7 @@
       </c>
       <c r="C46" s="2"/>
     </row>
-    <row r="47" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>41</v>
       </c>
@@ -1433,7 +1436,7 @@
       </c>
       <c r="C47" s="2"/>
     </row>
-    <row r="48" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="8" t="s">
         <v>6</v>
       </c>
@@ -1441,7 +1444,7 @@
       <c r="C48" s="8"/>
       <c r="D48" s="8"/>
     </row>
-    <row r="49" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>4</v>
       </c>
@@ -1450,7 +1453,7 @@
       </c>
       <c r="C49" s="2"/>
     </row>
-    <row r="50" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>3</v>
       </c>
@@ -1459,7 +1462,7 @@
       </c>
       <c r="C50" s="2"/>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>5</v>
       </c>
@@ -1468,7 +1471,7 @@
       </c>
       <c r="C51" s="2"/>
     </row>
-    <row r="52" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>21</v>
       </c>
@@ -1477,7 +1480,7 @@
       </c>
       <c r="C52" s="2"/>
     </row>
-    <row r="53" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>22</v>
       </c>
@@ -1486,7 +1489,7 @@
       </c>
       <c r="C53" s="2"/>
     </row>
-    <row r="54" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>23</v>
       </c>
@@ -1495,7 +1498,7 @@
       </c>
       <c r="C54" s="2"/>
     </row>
-    <row r="55" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
         <v>7</v>
       </c>
@@ -1503,7 +1506,7 @@
       <c r="C55" s="8"/>
       <c r="D55" s="8"/>
     </row>
-    <row r="56" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>4</v>
       </c>
@@ -1512,7 +1515,7 @@
       </c>
       <c r="C56" s="2"/>
     </row>
-    <row r="57" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>3</v>
       </c>
@@ -1521,7 +1524,7 @@
       </c>
       <c r="C57" s="2"/>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>5</v>
       </c>
@@ -1530,7 +1533,7 @@
       </c>
       <c r="C58" s="2"/>
     </row>
-    <row r="59" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>27</v>
       </c>
@@ -1539,7 +1542,7 @@
       </c>
       <c r="C59" s="2"/>
     </row>
-    <row r="60" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>28</v>
       </c>
@@ -1548,7 +1551,7 @@
       </c>
       <c r="C60" s="2"/>
     </row>
-    <row r="61" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>29</v>
       </c>
@@ -1557,7 +1560,7 @@
       </c>
       <c r="C61" s="2"/>
     </row>
-    <row r="62" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="8" t="s">
         <v>8</v>
       </c>
@@ -1565,7 +1568,7 @@
       <c r="C62" s="8"/>
       <c r="D62" s="8"/>
     </row>
-    <row r="63" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>4</v>
       </c>
@@ -1574,7 +1577,7 @@
       </c>
       <c r="C63" s="2"/>
     </row>
-    <row r="64" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>3</v>
       </c>
@@ -1583,7 +1586,7 @@
       </c>
       <c r="C64" s="2"/>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>5</v>
       </c>
@@ -1592,7 +1595,7 @@
       </c>
       <c r="C65" s="2"/>
     </row>
-    <row r="66" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>33</v>
       </c>
@@ -1603,7 +1606,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="67" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>34</v>
       </c>
@@ -1614,7 +1617,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="68" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>35</v>
       </c>
@@ -1625,7 +1628,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="69" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="8" t="s">
         <v>10</v>
       </c>
@@ -1633,7 +1636,7 @@
       <c r="C69" s="8"/>
       <c r="D69" s="8"/>
     </row>
-    <row r="70" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>4</v>
       </c>
@@ -1642,7 +1645,7 @@
       </c>
       <c r="C70" s="2"/>
     </row>
-    <row r="71" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>3</v>
       </c>
@@ -1651,7 +1654,7 @@
       </c>
       <c r="C71" s="2"/>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>5</v>
       </c>
@@ -1660,7 +1663,7 @@
       </c>
       <c r="C72" s="2"/>
     </row>
-    <row r="73" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>45</v>
       </c>
@@ -1669,7 +1672,7 @@
       </c>
       <c r="C73" s="2"/>
     </row>
-    <row r="74" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>46</v>
       </c>
@@ -1678,7 +1681,7 @@
       </c>
       <c r="C74" s="2"/>
     </row>
-    <row r="75" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>47</v>
       </c>
@@ -1687,7 +1690,7 @@
       </c>
       <c r="C75" s="2"/>
     </row>
-    <row r="76" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="8" t="s">
         <v>11</v>
       </c>
@@ -1695,7 +1698,7 @@
       <c r="C76" s="8"/>
       <c r="D76" s="8"/>
     </row>
-    <row r="77" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>4</v>
       </c>
@@ -1704,7 +1707,7 @@
       </c>
       <c r="C77" s="2"/>
     </row>
-    <row r="78" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>3</v>
       </c>
@@ -1713,7 +1716,7 @@
       </c>
       <c r="C78" s="2"/>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>5</v>
       </c>
@@ -1722,7 +1725,7 @@
       </c>
       <c r="C79" s="2"/>
     </row>
-    <row r="80" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>51</v>
       </c>
@@ -1731,7 +1734,7 @@
       </c>
       <c r="C80" s="2"/>
     </row>
-    <row r="81" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>52</v>
       </c>
@@ -1740,7 +1743,7 @@
       </c>
       <c r="C81" s="2"/>
     </row>
-    <row r="82" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>53</v>
       </c>
@@ -1749,15 +1752,15 @@
       </c>
       <c r="C82" s="2"/>
     </row>
-    <row r="83" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B83" s="8"/>
       <c r="C83" s="8"/>
       <c r="D83" s="8"/>
     </row>
-    <row r="84" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>4</v>
       </c>
@@ -1766,7 +1769,7 @@
       </c>
       <c r="C84" s="2"/>
     </row>
-    <row r="85" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>3</v>
       </c>
@@ -1775,7 +1778,7 @@
       </c>
       <c r="C85" s="2"/>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>5</v>
       </c>
@@ -1784,48 +1787,48 @@
       </c>
       <c r="C86" s="2"/>
     </row>
-    <row r="87" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C87" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="88" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="C88" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="89" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C89" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="90" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="8" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B90" s="8"/>
       <c r="C90" s="8"/>
       <c r="D90" s="8"/>
     </row>
-    <row r="91" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>4</v>
       </c>
@@ -1834,7 +1837,7 @@
       </c>
       <c r="C91" s="2"/>
     </row>
-    <row r="92" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>3</v>
       </c>
@@ -1843,7 +1846,7 @@
       </c>
       <c r="C92" s="2"/>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>5</v>
       </c>
@@ -1852,48 +1855,48 @@
       </c>
       <c r="C93" s="2"/>
     </row>
-    <row r="94" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C94" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="95" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C95" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="96" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C96" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="97" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B97" s="8"/>
       <c r="C97" s="8"/>
       <c r="D97" s="8"/>
     </row>
-    <row r="98" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>4</v>
       </c>
@@ -1902,7 +1905,7 @@
       </c>
       <c r="C98" s="2"/>
     </row>
-    <row r="99" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>3</v>
       </c>
@@ -1911,7 +1914,7 @@
       </c>
       <c r="C99" s="2"/>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>5</v>
       </c>
@@ -1920,48 +1923,48 @@
       </c>
       <c r="C100" s="2"/>
     </row>
-    <row r="101" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B101" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="B101" s="1" t="s">
-        <v>152</v>
-      </c>
       <c r="C101" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A102" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A103" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="8" t="s">
         <v>151</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A102" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="B102" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="C102" s="2" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A103" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="B103" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="C103" s="2" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A104" s="8" t="s">
-        <v>155</v>
       </c>
       <c r="B104" s="8"/>
       <c r="C104" s="8"/>
       <c r="D104" s="8"/>
     </row>
-    <row r="105" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>4</v>
       </c>
@@ -1970,7 +1973,7 @@
       </c>
       <c r="C105" s="2"/>
     </row>
-    <row r="106" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>3</v>
       </c>
@@ -1979,7 +1982,7 @@
       </c>
       <c r="C106" s="2"/>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>5</v>
       </c>
@@ -1988,48 +1991,48 @@
       </c>
       <c r="C107" s="2"/>
     </row>
-    <row r="108" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="C108" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="109" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C109" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="110" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C110" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="111" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="8" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B111" s="8"/>
       <c r="C111" s="8"/>
       <c r="D111" s="8"/>
     </row>
-    <row r="112" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>4</v>
       </c>
@@ -2038,7 +2041,7 @@
       </c>
       <c r="C112" s="2"/>
     </row>
-    <row r="113" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>3</v>
       </c>
@@ -2047,7 +2050,7 @@
       </c>
       <c r="C113" s="2"/>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>5</v>
       </c>
@@ -2056,48 +2059,48 @@
       </c>
       <c r="C114" s="2"/>
     </row>
-    <row r="115" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C115" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="116" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="C116" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="117" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C117" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="118" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="8" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B118" s="8"/>
       <c r="C118" s="8"/>
       <c r="D118" s="8"/>
     </row>
-    <row r="119" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>4</v>
       </c>
@@ -2106,7 +2109,7 @@
       </c>
       <c r="C119" s="2"/>
     </row>
-    <row r="120" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>3</v>
       </c>
@@ -2115,7 +2118,7 @@
       </c>
       <c r="C120" s="2"/>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>5</v>
       </c>
@@ -2124,42 +2127,42 @@
       </c>
       <c r="C121" s="2"/>
     </row>
-    <row r="122" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C122" s="2"/>
+    </row>
+    <row r="123" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A123" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B123" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B122" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="C122" s="2"/>
-    </row>
-    <row r="123" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A123" s="1" t="s">
+      <c r="C123" s="2"/>
+    </row>
+    <row r="124" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A124" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B124" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B123" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="C123" s="2"/>
-    </row>
-    <row r="124" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A124" s="1" t="s">
+      <c r="C124" s="2"/>
+    </row>
+    <row r="125" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A125" s="8" t="s">
         <v>166</v>
-      </c>
-      <c r="B124" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="C124" s="2"/>
-    </row>
-    <row r="125" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A125" s="8" t="s">
-        <v>170</v>
       </c>
       <c r="B125" s="8"/>
       <c r="C125" s="8"/>
       <c r="D125" s="8"/>
     </row>
-    <row r="126" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>4</v>
       </c>
@@ -2168,7 +2171,7 @@
       </c>
       <c r="C126" s="2"/>
     </row>
-    <row r="127" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>3</v>
       </c>
@@ -2177,7 +2180,7 @@
       </c>
       <c r="C127" s="2"/>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
         <v>5</v>
       </c>
@@ -2186,42 +2189,42 @@
       </c>
       <c r="C128" s="2"/>
     </row>
-    <row r="129" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C129" s="2"/>
+    </row>
+    <row r="130" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A130" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B130" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="B129" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="C129" s="2"/>
-    </row>
-    <row r="130" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A130" s="1" t="s">
+      <c r="C130" s="2"/>
+    </row>
+    <row r="131" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A131" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B131" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B130" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="C130" s="2"/>
-    </row>
-    <row r="131" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A131" s="1" t="s">
+      <c r="C131" s="2"/>
+    </row>
+    <row r="132" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A132" s="8" t="s">
         <v>173</v>
-      </c>
-      <c r="B131" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="C131" s="2"/>
-    </row>
-    <row r="132" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A132" s="8" t="s">
-        <v>177</v>
       </c>
       <c r="B132" s="8"/>
       <c r="C132" s="8"/>
       <c r="D132" s="8"/>
     </row>
-    <row r="133" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
         <v>4</v>
       </c>
@@ -2230,7 +2233,7 @@
       </c>
       <c r="C133" s="2"/>
     </row>
-    <row r="134" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
         <v>3</v>
       </c>
@@ -2239,7 +2242,7 @@
       </c>
       <c r="C134" s="2"/>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
         <v>5</v>
       </c>
@@ -2248,41 +2251,41 @@
       </c>
       <c r="C135" s="2"/>
     </row>
-    <row r="136" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B136" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="C136" s="2"/>
+    </row>
+    <row r="137" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A137" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B137" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="B136" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="C136" s="2"/>
-    </row>
-    <row r="137" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A137" s="1" t="s">
+      <c r="C137" s="2"/>
+    </row>
+    <row r="138" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A138" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="B138" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="B137" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="C137" s="2"/>
-    </row>
-    <row r="138" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A138" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="B138" s="1" t="s">
-        <v>183</v>
-      </c>
       <c r="C138" s="2"/>
     </row>
-    <row r="139" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="8" t="s">
         <v>73</v>
       </c>
       <c r="B139" s="8"/>
       <c r="C139" s="10"/>
     </row>
-    <row r="140" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
         <v>4</v>
       </c>
@@ -2291,7 +2294,7 @@
       </c>
       <c r="C140" s="2"/>
     </row>
-    <row r="141" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
         <v>3</v>
       </c>
@@ -2300,7 +2303,7 @@
       </c>
       <c r="C141" s="2"/>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
         <v>5</v>
       </c>
@@ -2309,7 +2312,7 @@
       </c>
       <c r="C142" s="2"/>
     </row>
-    <row r="143" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
         <v>74</v>
       </c>
@@ -2318,7 +2321,7 @@
       </c>
       <c r="C143" s="2"/>
     </row>
-    <row r="144" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
         <v>75</v>
       </c>
@@ -2327,25 +2330,29 @@
       </c>
       <c r="C144" s="2"/>
     </row>
-    <row r="145" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
         <v>76</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="C145" s="2"/>
-    </row>
-    <row r="146" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>200</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>77</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="C146" s="2"/>
-    </row>
-    <row r="147" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>201</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
         <v>78</v>
       </c>
@@ -2354,23 +2361,23 @@
       </c>
       <c r="C147" s="2"/>
     </row>
-    <row r="148" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
         <v>79</v>
       </c>
       <c r="B148" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C148" s="2"/>
+    </row>
+    <row r="149" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A149" s="8" t="s">
         <v>84</v>
-      </c>
-      <c r="C148" s="2"/>
-    </row>
-    <row r="149" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A149" s="8" t="s">
-        <v>86</v>
       </c>
       <c r="B149" s="8"/>
       <c r="C149" s="10"/>
     </row>
-    <row r="150" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
         <v>4</v>
       </c>
@@ -2379,7 +2386,7 @@
       </c>
       <c r="C150" s="2"/>
     </row>
-    <row r="151" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
         <v>3</v>
       </c>
@@ -2388,7 +2395,7 @@
       </c>
       <c r="C151" s="2"/>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
         <v>5</v>
       </c>
@@ -2397,61 +2404,65 @@
       </c>
       <c r="C152" s="2"/>
     </row>
-    <row r="153" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B153" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C153" s="2"/>
+    </row>
+    <row r="154" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A154" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B154" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C154" s="2"/>
+    </row>
+    <row r="155" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A155" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B153" s="1" t="s">
+      <c r="B155" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="C155" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A156" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B156" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C156" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A157" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B157" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="C153" s="2"/>
-    </row>
-    <row r="154" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A154" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B154" s="1" t="s">
+      <c r="C157" s="2"/>
+    </row>
+    <row r="158" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A158" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B158" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C154" s="2"/>
-    </row>
-    <row r="155" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A155" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="B155" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C155" s="2"/>
-    </row>
-    <row r="156" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A156" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B156" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C156" s="2"/>
-    </row>
-    <row r="157" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A157" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="B157" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="C157" s="2"/>
-    </row>
-    <row r="158" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A158" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B158" s="1" t="s">
-        <v>98</v>
-      </c>
       <c r="C158" s="2"/>
     </row>
-    <row r="159" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A159" s="8" t="s">
         <v>57</v>
       </c>
@@ -2459,7 +2470,7 @@
       <c r="C159" s="8"/>
       <c r="D159" s="8"/>
     </row>
-    <row r="160" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
         <v>4</v>
       </c>
@@ -2468,7 +2479,7 @@
       </c>
       <c r="C160" s="2"/>
     </row>
-    <row r="161" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
         <v>3</v>
       </c>
@@ -2477,7 +2488,7 @@
       </c>
       <c r="C161" s="2"/>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
         <v>5</v>
       </c>
@@ -2486,7 +2497,7 @@
       </c>
       <c r="C162" s="2"/>
     </row>
-    <row r="163" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
         <v>58</v>
       </c>
@@ -2495,7 +2506,7 @@
       </c>
       <c r="C163" s="2"/>
     </row>
-    <row r="164" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
         <v>60</v>
       </c>
@@ -2504,7 +2515,7 @@
       </c>
       <c r="C164" s="2"/>
     </row>
-    <row r="165" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="s">
         <v>59</v>
       </c>
@@ -2513,15 +2524,15 @@
       </c>
       <c r="C165" s="2"/>
     </row>
-    <row r="166" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A166" s="8" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B166" s="8"/>
       <c r="C166" s="8"/>
       <c r="D166" s="8"/>
     </row>
-    <row r="167" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
         <v>4</v>
       </c>
@@ -2530,7 +2541,7 @@
       </c>
       <c r="C167" s="2"/>
     </row>
-    <row r="168" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
         <v>3</v>
       </c>
@@ -2539,7 +2550,7 @@
       </c>
       <c r="C168" s="2"/>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="s">
         <v>5</v>
       </c>
@@ -2548,34 +2559,34 @@
       </c>
       <c r="C169" s="2"/>
     </row>
-    <row r="170" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="B170" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="C170" s="2"/>
+    </row>
+    <row r="171" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A171" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B171" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="B170" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="C170" s="2"/>
-    </row>
-    <row r="171" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A171" s="1" t="s">
+      <c r="C171" s="2"/>
+    </row>
+    <row r="172" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A172" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B172" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="B171" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="C171" s="2"/>
-    </row>
-    <row r="172" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A172" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="B172" s="1" t="s">
-        <v>190</v>
-      </c>
       <c r="C172" s="2"/>
     </row>
-    <row r="173" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A173" s="8" t="s">
         <v>61</v>
       </c>
@@ -2583,7 +2594,7 @@
       <c r="C173" s="8"/>
       <c r="D173" s="8"/>
     </row>
-    <row r="174" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="s">
         <v>4</v>
       </c>
@@ -2592,7 +2603,7 @@
       </c>
       <c r="C174" s="2"/>
     </row>
-    <row r="175" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A175" s="1" t="s">
         <v>3</v>
       </c>
@@ -2601,7 +2612,7 @@
       </c>
       <c r="C175" s="2"/>
     </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="1" t="s">
         <v>5</v>
       </c>
@@ -2610,7 +2621,7 @@
       </c>
       <c r="C176" s="2"/>
     </row>
-    <row r="177" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A177" s="1" t="s">
         <v>62</v>
       </c>
@@ -2619,7 +2630,7 @@
       </c>
       <c r="C177" s="2"/>
     </row>
-    <row r="178" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A178" s="1" t="s">
         <v>63</v>
       </c>
@@ -2628,7 +2639,7 @@
       </c>
       <c r="C178" s="2"/>
     </row>
-    <row r="179" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A179" s="1" t="s">
         <v>64</v>
       </c>
@@ -2637,15 +2648,15 @@
       </c>
       <c r="C179" s="2"/>
     </row>
-    <row r="180" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A180" s="8" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B180" s="8"/>
       <c r="C180" s="8"/>
       <c r="D180" s="8"/>
     </row>
-    <row r="181" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A181" s="1" t="s">
         <v>4</v>
       </c>
@@ -2654,7 +2665,7 @@
       </c>
       <c r="C181" s="2"/>
     </row>
-    <row r="182" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A182" s="1" t="s">
         <v>3</v>
       </c>
@@ -2663,7 +2674,7 @@
       </c>
       <c r="C182" s="2"/>
     </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" s="1" t="s">
         <v>5</v>
       </c>
@@ -2672,30 +2683,30 @@
       </c>
       <c r="C183" s="2"/>
     </row>
-    <row r="184" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A184" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B184" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C184" s="2"/>
+    </row>
+    <row r="185" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A185" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B185" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="B184" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="C184" s="2"/>
-    </row>
-    <row r="185" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A185" s="1" t="s">
+      <c r="C185" s="2"/>
+    </row>
+    <row r="186" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A186" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B186" s="1" t="s">
         <v>193</v>
-      </c>
-      <c r="B185" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="C185" s="2"/>
-    </row>
-    <row r="186" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A186" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="B186" s="1" t="s">
-        <v>197</v>
       </c>
       <c r="C186" s="2"/>
     </row>

</xml_diff>